<commit_message>
Connect Coding Questions to ConceptNodes
</commit_message>
<xml_diff>
--- a/server_nestjs/src/storage/wise2324_OFP_workshop_aufgaben.xlsx
+++ b/server_nestjs/src/storage/wise2324_OFP_workshop_aufgaben.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10114"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Tutor-Kai\server_nestjs\src\storage\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcsauer/GitHub/hefl/server_nestjs/src/storage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82ABE88D-1C38-45B0-930A-A0AE3A1252E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72ADF046-1E6E-FD4C-AC66-F86B7AE52965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15320" yWindow="740" windowWidth="14920" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="290">
   <si>
     <t>Test</t>
   </si>
@@ -3646,6 +3646,9 @@
 &lt;em&gt;[(&amp;#39;s&amp;#39;, 4), (&amp;#39;t&amp;#39;, 4), (&amp;#39;i&amp;#39;, 3), (&amp;#39;e&amp;#39;, 2), (&amp;#39;n&amp;#39;, 2), (&amp;#39;d&amp;#39;, 1), (&amp;#39;a&amp;#39;, 1), (&amp;#39;r&amp;#39;, 1), (&amp;#39;g&amp;#39;, 1)]&lt;/em&gt;&lt;br /&gt;
 &lt;br /&gt;
 &amp;nbsp;</t>
+  </si>
+  <si>
+    <t>ConceptNodeID</t>
   </si>
 </sst>
 </file>
@@ -4014,20 +4017,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:P39"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="23.08984375" customWidth="1"/>
-    <col min="4" max="4" width="37.08984375" customWidth="1"/>
-    <col min="5" max="5" width="66.6328125" customWidth="1"/>
-    <col min="6" max="6" width="143.08984375" customWidth="1"/>
-    <col min="7" max="7" width="105.54296875" customWidth="1"/>
-    <col min="8" max="8" width="23.6328125" customWidth="1"/>
-    <col min="10" max="10" width="49.90625" customWidth="1"/>
-    <col min="11" max="11" width="74.54296875" customWidth="1"/>
+    <col min="3" max="4" width="23.1640625" customWidth="1"/>
+    <col min="5" max="5" width="37.1640625" customWidth="1"/>
+    <col min="6" max="6" width="66.6640625" customWidth="1"/>
+    <col min="7" max="7" width="143.1640625" customWidth="1"/>
+    <col min="8" max="8" width="105.5" customWidth="1"/>
+    <col min="9" max="9" width="23.6640625" customWidth="1"/>
+    <col min="11" max="11" width="49.83203125" customWidth="1"/>
+    <col min="12" max="12" width="74.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -4038,25 +4041,28 @@
         <v>201</v>
       </c>
       <c r="D1" t="s">
+        <v>289</v>
+      </c>
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>24</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>54</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4066,32 +4072,35 @@
       <c r="C2" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2">
+        <v>34</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="I2" s="2">
+      <c r="J2" s="2">
         <v>0</v>
       </c>
-      <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
-    </row>
-    <row r="3" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P2" s="2"/>
+    </row>
+    <row r="3" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4101,32 +4110,35 @@
       <c r="C3" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2">
+        <v>36</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J3" s="2">
         <v>0</v>
       </c>
-      <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
-    </row>
-    <row r="4" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P3" s="2"/>
+    </row>
+    <row r="4" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -4136,32 +4148,35 @@
       <c r="C4" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2">
+        <v>34</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="I4" s="2">
+      <c r="J4" s="2">
         <v>0</v>
       </c>
-      <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
-    </row>
-    <row r="5" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P4" s="2"/>
+    </row>
+    <row r="5" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -4171,32 +4186,35 @@
       <c r="C5" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="2">
+        <v>34</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="I5" s="2">
+      <c r="J5" s="2">
         <v>0</v>
       </c>
-      <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-    </row>
-    <row r="6" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P5" s="2"/>
+    </row>
+    <row r="6" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -4206,32 +4224,35 @@
       <c r="C6" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="2">
+        <v>52</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="I6" s="2">
+      <c r="J6" s="2">
         <v>0</v>
       </c>
-      <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
-    </row>
-    <row r="7" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P6" s="2"/>
+    </row>
+    <row r="7" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -4241,32 +4262,35 @@
       <c r="C7" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="2">
+        <v>34</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="I7" s="2">
+      <c r="J7" s="2">
         <v>0</v>
       </c>
-      <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
-    </row>
-    <row r="8" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P7" s="2"/>
+    </row>
+    <row r="8" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -4276,32 +4300,35 @@
       <c r="C8" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="2">
+        <v>34</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I8" s="2">
+      <c r="J8" s="2">
         <v>0</v>
       </c>
-      <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-    </row>
-    <row r="9" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P8" s="2"/>
+    </row>
+    <row r="9" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -4311,32 +4338,35 @@
       <c r="C9" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="2">
+        <v>26</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="I9" s="2">
+      <c r="J9" s="2">
         <v>0</v>
       </c>
-      <c r="J9" s="2"/>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-    </row>
-    <row r="10" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P9" s="2"/>
+    </row>
+    <row r="10" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -4346,32 +4376,35 @@
       <c r="C10" t="s">
         <v>253</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="2">
+        <v>63</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="I10" s="2">
+      <c r="J10" s="2">
         <v>0</v>
       </c>
-      <c r="J10" s="2"/>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
-    </row>
-    <row r="11" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P10" s="2"/>
+    </row>
+    <row r="11" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -4381,32 +4414,35 @@
       <c r="C11" t="s">
         <v>253</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="2">
+        <v>65</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I11" s="2">
+      <c r="J11" s="2">
         <v>0</v>
       </c>
-      <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
-    </row>
-    <row r="12" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P11" s="2"/>
+    </row>
+    <row r="12" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -4416,32 +4452,35 @@
       <c r="C12" t="s">
         <v>253</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="2">
+        <v>63</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="I12" s="2">
+      <c r="J12" s="2">
         <v>1</v>
       </c>
-      <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
-    </row>
-    <row r="13" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P12" s="2"/>
+    </row>
+    <row r="13" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -4451,32 +4490,35 @@
       <c r="C13" t="s">
         <v>253</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="2">
+        <v>63</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="I13" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="I13" s="2">
+      <c r="J13" s="2">
         <v>0</v>
       </c>
-      <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
-    </row>
-    <row r="14" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P13" s="2"/>
+    </row>
+    <row r="14" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -4486,26 +4528,29 @@
       <c r="C14" t="s">
         <v>253</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="2">
+        <v>69</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>62</v>
       </c>
-      <c r="I14" s="2">
+      <c r="J14" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -4515,26 +4560,29 @@
       <c r="C15" t="s">
         <v>253</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="2">
+        <v>70</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="G15" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="H15" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>64</v>
       </c>
-      <c r="I15" s="2">
+      <c r="J15" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -4544,26 +4592,29 @@
       <c r="C16" t="s">
         <v>253</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="2">
+        <v>64</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G16" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="H16" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>65</v>
       </c>
-      <c r="I16" s="2">
+      <c r="J16" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -4573,26 +4624,29 @@
       <c r="C17" t="s">
         <v>253</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="2">
+        <v>74</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="F17" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="H17" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="I17" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="I17" s="2">
+      <c r="J17" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -4602,26 +4656,29 @@
       <c r="C18" t="s">
         <v>253</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="2">
+        <v>84</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="G18" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>95</v>
       </c>
-      <c r="I18" s="2">
+      <c r="J18" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -4631,26 +4688,29 @@
       <c r="C19" t="s">
         <v>253</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="2">
+        <v>93</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="G19" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="H19" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>100</v>
       </c>
-      <c r="I19" s="2">
+      <c r="J19" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -4660,26 +4720,29 @@
       <c r="C20" t="s">
         <v>253</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="2">
+        <v>69</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="F20" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="G20" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="H20" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="I20" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="I20" s="2">
+      <c r="J20" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -4689,26 +4752,29 @@
       <c r="C21" t="s">
         <v>253</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="2">
+        <v>78</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="G21" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="H21" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>136</v>
       </c>
-      <c r="I21" s="2">
+      <c r="J21" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -4718,26 +4784,29 @@
       <c r="C22" t="s">
         <v>253</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="2">
+        <v>74</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="F22" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="G22" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="H22" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="I22" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="I22" s="2">
+      <c r="J22" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -4747,26 +4816,29 @@
       <c r="C23" t="s">
         <v>253</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="2">
+        <v>78</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="F23" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="G23" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="H23" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="I23" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="I23" s="2">
+      <c r="J23" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -4776,26 +4848,29 @@
       <c r="C24" t="s">
         <v>253</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="F24" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="G24" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="H24" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="I24" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="I24" s="2">
+      <c r="J24" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -4805,26 +4880,29 @@
       <c r="C25" t="s">
         <v>253</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="2">
+        <v>1</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="F25" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="G25" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="H25" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="I25" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="I25" s="2">
+      <c r="J25" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -4834,26 +4912,29 @@
       <c r="C26" t="s">
         <v>253</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="2">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="F26" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="G26" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="H26" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="I26" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="I26" s="2">
+      <c r="J26" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -4863,26 +4944,29 @@
       <c r="C27" t="s">
         <v>253</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="2">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="F27" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="G27" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="H27" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="I27" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="I27" s="2">
+      <c r="J27" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -4892,26 +4976,29 @@
       <c r="C28" t="s">
         <v>253</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="2">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="F28" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="G28" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="H28" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="I28" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="I28" s="2">
+      <c r="J28" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -4921,32 +5008,35 @@
       <c r="C29" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="2">
+        <v>40</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="G29" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="G29" s="1" t="s">
+      <c r="H29" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="I29" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="I29" s="2">
+      <c r="J29" s="2">
         <v>0</v>
       </c>
-      <c r="J29" s="1" t="s">
+      <c r="K29" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="K29" s="1" t="s">
+      <c r="L29" s="1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -4956,32 +5046,35 @@
       <c r="C30" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="2">
+        <v>26</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="I30" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="I30" s="2">
+      <c r="J30" s="2">
         <v>0</v>
       </c>
-      <c r="J30" s="1" t="s">
+      <c r="K30" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="K30" s="1" t="s">
+      <c r="L30" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -4991,32 +5084,35 @@
       <c r="C31" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="2">
+        <v>34</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="I31" s="2">
+      <c r="J31" s="2">
         <v>0</v>
       </c>
-      <c r="J31" s="1" t="s">
+      <c r="K31" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="K31" s="1" t="s">
+      <c r="L31" s="1" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -5026,32 +5122,35 @@
       <c r="C32" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="2">
+        <v>34</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="F32" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="G32" s="1" t="s">
+      <c r="H32" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="I32" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="I32" s="2">
+      <c r="J32" s="2">
         <v>0</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="K32" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="K32" s="1" t="s">
+      <c r="L32" s="1" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -5061,32 +5160,35 @@
       <c r="C33" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="2">
+        <v>26</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="G33" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="H33" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="I33" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="I33" s="2">
+      <c r="J33" s="2">
         <v>0</v>
       </c>
-      <c r="J33" s="1" t="s">
+      <c r="K33" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="K33" s="1" t="s">
+      <c r="L33" s="1" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -5096,32 +5198,35 @@
       <c r="C34" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="2">
+        <v>28</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="G34" s="1" t="s">
+      <c r="H34" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="I34" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="I34" s="2">
+      <c r="J34" s="2">
         <v>0</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="K34" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="K34" s="1" t="s">
+      <c r="L34" s="1" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -5131,32 +5236,35 @@
       <c r="C35" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D35" s="2">
+        <v>26</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="G35" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="G35" s="1" t="s">
+      <c r="H35" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="I35" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="I35" s="2">
+      <c r="J35" s="2">
         <v>0</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="K35" s="1" t="s">
+      <c r="L35" s="1" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -5166,32 +5274,35 @@
       <c r="C36" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D36" s="2">
+        <v>34</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="F36" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="G36" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="G36" s="1" t="s">
+      <c r="H36" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="I36" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="I36" s="2">
+      <c r="J36" s="2">
         <v>0</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="K36" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="K36" s="1" t="s">
+      <c r="L36" s="1" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -5201,32 +5312,35 @@
       <c r="C37" t="s">
         <v>253</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D37" s="2">
+        <v>1</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="F37" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="I37" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="I37" s="2">
+      <c r="J37" s="2">
         <v>0</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="K37" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="K37" s="1" t="s">
+      <c r="L37" s="1" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -5236,32 +5350,35 @@
       <c r="C38" t="s">
         <v>253</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="D38" s="2">
+        <v>1</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="F38" s="8" t="s">
         <v>271</v>
       </c>
-      <c r="F38" s="8" t="s">
+      <c r="G38" s="8" t="s">
         <v>275</v>
       </c>
-      <c r="G38" s="8" t="s">
+      <c r="H38" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="H38" t="s">
+      <c r="I38" t="s">
         <v>272</v>
       </c>
-      <c r="I38" s="2">
+      <c r="J38" s="2">
         <v>0</v>
       </c>
-      <c r="J38" s="4" t="s">
+      <c r="K38" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="K38" s="4" t="s">
+      <c r="L38" s="4" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -5271,28 +5388,31 @@
       <c r="C39" t="s">
         <v>253</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="D39" s="2">
+        <v>1</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="F39" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="G39" s="4" t="s">
         <v>279</v>
       </c>
-      <c r="G39" s="4" t="s">
+      <c r="H39" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="H39" s="4" t="s">
+      <c r="I39" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="I39" s="2">
+      <c r="J39" s="2">
         <v>0</v>
       </c>
-      <c r="J39" t="s">
+      <c r="K39" t="s">
         <v>245</v>
       </c>
-      <c r="K39" s="4" t="s">
+      <c r="L39" s="4" t="s">
         <v>251</v>
       </c>
     </row>
@@ -5305,13 +5425,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EB41A74-2920-4D11-8A4B-E3642DEC7AD7}">
   <dimension ref="A1:D63"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="27.36328125" customWidth="1"/>
-    <col min="4" max="4" width="129.6328125" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" customWidth="1"/>
+    <col min="4" max="4" width="129.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>50</v>
       </c>
@@ -5325,7 +5445,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>ROW()-1</f>
         <v>1</v>
@@ -5340,7 +5460,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3">
         <f>ROW()-1</f>
         <v>2</v>
@@ -5355,7 +5475,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4">
         <f>ROW()-1</f>
         <v>3</v>
@@ -5370,7 +5490,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5">
         <f t="shared" ref="A5:A27" si="0">ROW()-1</f>
         <v>4</v>
@@ -5385,7 +5505,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -5400,7 +5520,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -5415,7 +5535,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -5430,7 +5550,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -5445,7 +5565,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="180.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="196" x14ac:dyDescent="0.2">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -5460,7 +5580,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -5475,7 +5595,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="240.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="261" x14ac:dyDescent="0.2">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -5490,7 +5610,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="168.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="183" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -5505,7 +5625,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="204.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" ht="222" x14ac:dyDescent="0.2">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -5520,7 +5640,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="252.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" ht="273" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -5535,7 +5655,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="228.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" ht="248" x14ac:dyDescent="0.2">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -5550,7 +5670,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -5565,7 +5685,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -5580,7 +5700,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -5595,7 +5715,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -5610,7 +5730,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -5625,7 +5745,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="180.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" ht="196" x14ac:dyDescent="0.2">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -5640,7 +5760,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -5655,7 +5775,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -5670,7 +5790,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -5685,7 +5805,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -5700,7 +5820,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -5715,7 +5835,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -5729,7 +5849,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="84.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" ht="92" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -5743,7 +5863,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -5757,7 +5877,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="84.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" ht="92" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -5771,7 +5891,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -5785,7 +5905,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="84.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" ht="92" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -5799,7 +5919,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="36.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" ht="40" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -5813,7 +5933,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="84.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" ht="92" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -5827,7 +5947,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -5841,7 +5961,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -5855,7 +5975,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" ht="112" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -5869,7 +5989,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -5883,7 +6003,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -5897,7 +6017,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -5911,7 +6031,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -5925,7 +6045,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -5939,7 +6059,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -5953,7 +6073,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" ht="176" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -5967,7 +6087,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -5981,7 +6101,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -5995,7 +6115,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -6009,7 +6129,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -6023,7 +6143,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -6037,7 +6157,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" ht="80" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -6051,7 +6171,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -6065,7 +6185,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" ht="32" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -6079,7 +6199,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -6093,7 +6213,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" ht="48" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -6107,7 +6227,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -6121,7 +6241,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -6135,7 +6255,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -6149,7 +6269,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -6163,7 +6283,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="116" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" ht="128" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -6177,7 +6297,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="232" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" ht="256" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -6191,7 +6311,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -6205,7 +6325,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>

</xml_diff>